<commit_message>
feat: add Excel basics, navigation, formatting, formulas, and cell referencing
</commit_message>
<xml_diff>
--- a/Excel/Excel-Practice.xlsx
+++ b/Excel/Excel-Practice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sankp\Downloads\python\Data-Analysis-And-Dashboards\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42FBFFFE-C7D3-4FD6-A74F-9B5DB5CD6D80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F47851A-A755-4A4E-AEF3-EDEA533152DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1208E387-7D59-452B-A9FE-4019E33F8484}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>ID</t>
   </si>
@@ -50,13 +50,73 @@
     <t xml:space="preserve">City </t>
   </si>
   <si>
-    <t>Region</t>
-  </si>
-  <si>
     <t>Salary</t>
   </si>
   <si>
     <t>Employee Data</t>
+  </si>
+  <si>
+    <t>Ram</t>
+  </si>
+  <si>
+    <t>Shyam</t>
+  </si>
+  <si>
+    <t>Prem</t>
+  </si>
+  <si>
+    <t>Karan</t>
+  </si>
+  <si>
+    <t>Arjun</t>
+  </si>
+  <si>
+    <t>Pranav</t>
+  </si>
+  <si>
+    <t>Shantanu</t>
+  </si>
+  <si>
+    <t>Pranay</t>
+  </si>
+  <si>
+    <t>Rama</t>
+  </si>
+  <si>
+    <t>Rudra</t>
+  </si>
+  <si>
+    <t>Kolhapur</t>
+  </si>
+  <si>
+    <t>Pune</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>Sangli</t>
+  </si>
+  <si>
+    <t>Satara</t>
+  </si>
+  <si>
+    <t>Expense Percentage</t>
+  </si>
+  <si>
+    <t>Net Salary</t>
+  </si>
+  <si>
+    <t>AVG Expenses</t>
+  </si>
+  <si>
+    <t>AVG Salary</t>
+  </si>
+  <si>
+    <t>AVG Net Salary</t>
   </si>
 </sst>
 </file>
@@ -459,19 +519,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6172E3A2-32EF-4915-A3C8-BDFED8837A01}">
-  <dimension ref="A2:E3"/>
+  <dimension ref="A2:F17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -482,10 +551,248 @@
         <v>2</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>15000</v>
+      </c>
+      <c r="F4">
+        <f>$E4-(($E4/100)*$D4)</f>
+        <v>13500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>20</v>
+      </c>
+      <c r="E5">
+        <v>20000</v>
+      </c>
+      <c r="F5">
+        <f>$E5-((E5/100)*$D5)</f>
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6">
+        <v>25</v>
+      </c>
+      <c r="E6">
+        <v>25000</v>
+      </c>
+      <c r="F6">
+        <f t="shared" ref="F5:F13" si="0">$E6-(($E6/100)*$D6)</f>
+        <v>18750</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
         <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7">
+        <v>30</v>
+      </c>
+      <c r="E7">
+        <v>12000</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="0"/>
+        <v>8400</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8">
+        <v>12</v>
+      </c>
+      <c r="E8">
+        <v>35000</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>30800</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>50000</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10">
+        <v>20</v>
+      </c>
+      <c r="E10">
+        <v>20000</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="0"/>
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11">
+        <v>20</v>
+      </c>
+      <c r="E11">
+        <v>22000</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="0"/>
+        <v>17600</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>9</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12">
+        <v>15</v>
+      </c>
+      <c r="E12">
+        <v>12000</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="0"/>
+        <v>10200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13">
+        <v>15</v>
+      </c>
+      <c r="E13">
+        <v>23000</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>19550</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D16" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="4:6" x14ac:dyDescent="0.3">
+      <c r="D17">
+        <f>AVERAGE(D4:D13)</f>
+        <v>17.7</v>
+      </c>
+      <c r="E17">
+        <f>AVERAGE(E4:E13)</f>
+        <v>23400</v>
+      </c>
+      <c r="F17">
+        <f>AVERAGE(F4:F13)</f>
+        <v>19580</v>
       </c>
     </row>
   </sheetData>

</xml_diff>